<commit_message>
Major UI revisions, better clarity and broader view of tables. Excel generation and pdf restrictions functionality done. User restrictions also updated.
</commit_message>
<xml_diff>
--- a/users.xlsx
+++ b/users.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -513,6 +513,28 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>2026-04-25 23:01:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>winstone</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>504aa67206a83ec5457c01d7abf122a7bd7dc4be4b58ede1339e45d25edf37df</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>user</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>2026-04-26 08:11:07</t>
         </is>
       </c>
     </row>

</xml_diff>